<commit_message>
Tambah referensi manual: 695176
</commit_message>
<xml_diff>
--- a/templates/Template_Data_Referensi.xlsx
+++ b/templates/Template_Data_Referensi.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data Referensi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,8 +464,10 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
-        <v>152</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -492,8 +494,10 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
-        <v>25</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -520,8 +524,10 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
-        <v>115</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -548,8 +554,10 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
-        <v>25</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -576,8 +584,10 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
-        <v>25</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -604,8 +614,10 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="n">
-        <v>12</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -634,8 +646,10 @@
       <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="n">
-        <v>66</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -662,8 +676,10 @@
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="n">
-        <v>56</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -690,8 +706,10 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="n">
-        <v>25</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -718,8 +736,10 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="n">
-        <v>25</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -746,8 +766,10 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="n">
-        <v>115</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -774,8 +796,10 @@
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="n">
-        <v>25</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -802,8 +826,10 @@
       <c r="A14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="n">
-        <v>56</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -830,8 +856,10 @@
       <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="n">
-        <v>5</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -858,8 +886,10 @@
       <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="n">
-        <v>25</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -886,8 +916,10 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="n">
-        <v>25</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -914,8 +946,10 @@
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="n">
-        <v>25</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -942,8 +976,10 @@
       <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="n">
-        <v>137</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -970,8 +1006,10 @@
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="n">
-        <v>25</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -998,8 +1036,10 @@
       <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="n">
-        <v>25</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1026,8 +1066,10 @@
       <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="n">
-        <v>137</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1054,8 +1096,10 @@
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="n">
-        <v>137</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1082,8 +1126,10 @@
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="n">
-        <v>5</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1110,8 +1156,10 @@
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="n">
-        <v>24</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1138,8 +1186,10 @@
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="n">
-        <v>6</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1166,8 +1216,10 @@
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="n">
-        <v>6</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1194,8 +1246,10 @@
       <c r="A28" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="n">
-        <v>25</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1222,8 +1276,10 @@
       <c r="A29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="n">
-        <v>25</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1250,8 +1306,10 @@
       <c r="A30" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="n">
-        <v>25</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1278,8 +1336,10 @@
       <c r="A31" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="n">
-        <v>6</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1306,8 +1366,10 @@
       <c r="A32" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="n">
-        <v>25</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1334,8 +1396,10 @@
       <c r="A33" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="n">
-        <v>25</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1362,8 +1426,10 @@
       <c r="A34" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="n">
-        <v>60</v>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1390,8 +1456,10 @@
       <c r="A35" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="n">
-        <v>25</v>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1418,8 +1486,10 @@
       <c r="A36" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="n">
-        <v>25</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1446,8 +1516,10 @@
       <c r="A37" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="n">
-        <v>76</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1474,8 +1546,10 @@
       <c r="A38" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="n">
-        <v>25</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1502,8 +1576,10 @@
       <c r="A39" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="n">
-        <v>25</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1530,8 +1606,10 @@
       <c r="A40" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="n">
-        <v>76</v>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1558,8 +1636,10 @@
       <c r="A41" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="n">
-        <v>12</v>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1586,8 +1666,10 @@
       <c r="A42" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="n">
-        <v>56</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1614,8 +1696,10 @@
       <c r="A43" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="n">
-        <v>25</v>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1642,8 +1726,10 @@
       <c r="A44" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="n">
-        <v>25</v>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1670,8 +1756,10 @@
       <c r="A45" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="n">
-        <v>25</v>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1698,8 +1786,10 @@
       <c r="A46" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="n">
-        <v>25</v>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1726,8 +1816,10 @@
       <c r="A47" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="n">
-        <v>25</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1754,8 +1846,10 @@
       <c r="A48" t="n">
         <v>47</v>
       </c>
-      <c r="B48" t="n">
-        <v>76</v>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1782,8 +1876,10 @@
       <c r="A49" t="n">
         <v>48</v>
       </c>
-      <c r="B49" t="n">
-        <v>5</v>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1810,8 +1906,10 @@
       <c r="A50" t="n">
         <v>49</v>
       </c>
-      <c r="B50" t="n">
-        <v>60</v>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1838,8 +1936,10 @@
       <c r="A51" t="n">
         <v>50</v>
       </c>
-      <c r="B51" t="n">
-        <v>25</v>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1866,8 +1966,10 @@
       <c r="A52" t="n">
         <v>51</v>
       </c>
-      <c r="B52" t="n">
-        <v>25</v>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1894,8 +1996,10 @@
       <c r="A53" t="n">
         <v>52</v>
       </c>
-      <c r="B53" t="n">
-        <v>137</v>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1922,8 +2026,10 @@
       <c r="A54" t="n">
         <v>53</v>
       </c>
-      <c r="B54" t="n">
-        <v>25</v>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1950,8 +2056,10 @@
       <c r="A55" t="n">
         <v>54</v>
       </c>
-      <c r="B55" t="n">
-        <v>25</v>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1978,8 +2086,10 @@
       <c r="A56" t="n">
         <v>55</v>
       </c>
-      <c r="B56" t="n">
-        <v>5</v>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -2006,8 +2116,10 @@
       <c r="A57" t="n">
         <v>56</v>
       </c>
-      <c r="B57" t="n">
-        <v>5</v>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -2034,8 +2146,10 @@
       <c r="A58" t="n">
         <v>57</v>
       </c>
-      <c r="B58" t="n">
-        <v>5</v>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -2062,8 +2176,10 @@
       <c r="A59" t="n">
         <v>58</v>
       </c>
-      <c r="B59" t="n">
-        <v>5</v>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -2090,8 +2206,10 @@
       <c r="A60" t="n">
         <v>59</v>
       </c>
-      <c r="B60" t="n">
-        <v>5</v>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -2118,8 +2236,10 @@
       <c r="A61" t="n">
         <v>60</v>
       </c>
-      <c r="B61" t="n">
-        <v>15</v>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -2146,8 +2266,10 @@
       <c r="A62" t="n">
         <v>61</v>
       </c>
-      <c r="B62" t="n">
-        <v>54</v>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -2174,8 +2296,10 @@
       <c r="A63" t="n">
         <v>62</v>
       </c>
-      <c r="B63" t="n">
-        <v>25</v>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -2202,8 +2326,10 @@
       <c r="A64" t="n">
         <v>63</v>
       </c>
-      <c r="B64" t="n">
-        <v>25</v>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -2230,8 +2356,10 @@
       <c r="A65" t="n">
         <v>64</v>
       </c>
-      <c r="B65" t="n">
-        <v>15</v>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -2258,8 +2386,10 @@
       <c r="A66" t="n">
         <v>65</v>
       </c>
-      <c r="B66" t="n">
-        <v>60</v>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -2286,8 +2416,10 @@
       <c r="A67" t="n">
         <v>66</v>
       </c>
-      <c r="B67" t="n">
-        <v>54</v>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -2314,8 +2446,10 @@
       <c r="A68" t="n">
         <v>67</v>
       </c>
-      <c r="B68" t="n">
-        <v>54</v>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -2342,8 +2476,10 @@
       <c r="A69" t="n">
         <v>68</v>
       </c>
-      <c r="B69" t="n">
-        <v>137</v>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -2370,8 +2506,10 @@
       <c r="A70" t="n">
         <v>70</v>
       </c>
-      <c r="B70" t="n">
-        <v>137</v>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2398,8 +2536,10 @@
       <c r="A71" t="n">
         <v>71</v>
       </c>
-      <c r="B71" t="n">
-        <v>137</v>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2426,8 +2566,10 @@
       <c r="A72" t="n">
         <v>72</v>
       </c>
-      <c r="B72" t="n">
-        <v>137</v>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2454,8 +2596,10 @@
       <c r="A73" t="n">
         <v>73</v>
       </c>
-      <c r="B73" t="n">
-        <v>137</v>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2482,8 +2626,10 @@
       <c r="A74" t="n">
         <v>74</v>
       </c>
-      <c r="B74" t="n">
-        <v>137</v>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2510,8 +2656,10 @@
       <c r="A75" t="n">
         <v>75</v>
       </c>
-      <c r="B75" t="n">
-        <v>24</v>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2538,8 +2686,10 @@
       <c r="A76" t="n">
         <v>76</v>
       </c>
-      <c r="B76" t="n">
-        <v>25</v>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2566,8 +2716,10 @@
       <c r="A77" t="n">
         <v>77</v>
       </c>
-      <c r="B77" t="n">
-        <v>25</v>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2594,8 +2746,10 @@
       <c r="A78" t="n">
         <v>78</v>
       </c>
-      <c r="B78" t="n">
-        <v>76</v>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2615,6 +2769,36 @@
       <c r="F78" t="inlineStr">
         <is>
           <t>KPU KABUPATEN PENUKAL ABAB LEMATANG ILIR</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>79</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>KEMENTERIAN HAJI DAN UMRAH</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>695176</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>KANTOR KEMENHAJ OKU</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>KANTOR KEMENTERIAN HAJI DAN UMRAH KAB. OGAN KOMERING ULU</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tambah referensi manual: 695182
</commit_message>
<xml_diff>
--- a/templates/Template_Data_Referensi.xlsx
+++ b/templates/Template_Data_Referensi.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2802,6 +2802,36 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>80</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>KEMENTERIAN HAJI DAN UMRAH</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>695182</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>KANTOR KEMENHAJ OKUT</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>KANTOR KEMENTERIAN HAJI DAN UMRAH KAB. OGAN KOMERING ULU TIMUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tambah referensi manual: 695184
</commit_message>
<xml_diff>
--- a/templates/Template_Data_Referensi.xlsx
+++ b/templates/Template_Data_Referensi.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2832,6 +2832,36 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>81</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>KEMENTERIAN HAJI DAN UMRAH</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>695184</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>KANTOR KEMENHAJ OKUS</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>KANTOR KEMENTERIAN HAJI DAN UMRAH KAB. OGAN KOMERING ULU SELATAN</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>